<commit_message>
Changes as per frontend, fixed bug for planned SKUs, utlization, efficiency
</commit_message>
<xml_diff>
--- a/load_cycle_times.xlsx
+++ b/load_cycle_times.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,12 +417,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>SKUCode</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>CycleTime_min</t>
         </is>
@@ -447,7 +435,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +445,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -467,7 +455,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -477,7 +465,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -487,7 +475,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -497,7 +485,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -507,7 +495,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -517,7 +505,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -527,7 +515,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
@@ -537,7 +525,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -547,7 +535,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -557,7 +545,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -567,7 +555,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
@@ -577,7 +565,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">
@@ -587,7 +575,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17">
@@ -597,7 +585,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18">
@@ -607,7 +595,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19">
@@ -617,7 +605,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20">
@@ -627,7 +615,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21">
@@ -637,7 +625,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22">
@@ -647,7 +635,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23">
@@ -677,7 +665,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26">
@@ -687,7 +675,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27">
@@ -697,7 +685,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28">
@@ -707,7 +695,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29">
@@ -717,7 +705,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30">
@@ -727,7 +715,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31">
@@ -737,7 +725,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32">
@@ -747,7 +735,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33">
@@ -767,7 +755,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35">
@@ -777,7 +765,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="36">
@@ -787,7 +775,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="37">
@@ -797,7 +785,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38">
@@ -807,7 +795,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="39">
@@ -817,7 +805,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="40">
@@ -827,7 +815,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41">
@@ -837,7 +825,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="42">
@@ -857,7 +845,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44">
@@ -867,7 +855,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="45">
@@ -877,7 +865,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="46">
@@ -887,7 +875,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="47">
@@ -897,7 +885,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="48">
@@ -907,7 +895,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="49">
@@ -917,7 +905,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="50">
@@ -927,7 +915,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="51">
@@ -937,7 +925,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="52">
@@ -957,7 +945,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="54">
@@ -967,7 +955,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="55">
@@ -977,7 +965,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="56">
@@ -987,7 +975,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="57">
@@ -1007,7 +995,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="59">
@@ -1017,7 +1005,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="60">
@@ -1027,7 +1015,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="61">
@@ -1077,7 +1065,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="66">
@@ -1087,7 +1075,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="67">
@@ -1097,7 +1085,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="68">
@@ -1107,7 +1095,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="69">
@@ -1147,7 +1135,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="73">
@@ -1157,7 +1145,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="74">
@@ -1167,7 +1155,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="75">
@@ -1177,7 +1165,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="76">
@@ -1187,7 +1175,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="77">
@@ -1197,7 +1185,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="78">
@@ -1207,7 +1195,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="79">
@@ -1217,7 +1205,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="80">
@@ -1227,7 +1215,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="81">
@@ -1237,7 +1225,7 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="82">
@@ -1247,7 +1235,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="83">
@@ -1257,7 +1245,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="84">
@@ -1267,7 +1255,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="85">
@@ -1277,7 +1265,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="86">
@@ -1287,7 +1275,7 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="87">
@@ -1297,7 +1285,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="88">
@@ -1307,7 +1295,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="89">
@@ -1317,7 +1305,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="90">
@@ -1337,7 +1325,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="92">
@@ -1347,7 +1335,7 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="93">
@@ -1357,7 +1345,7 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="94">
@@ -1367,7 +1355,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="95">
@@ -1397,7 +1385,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="98">
@@ -1407,7 +1395,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="99">
@@ -1417,7 +1405,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="100">
@@ -1427,7 +1415,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="101">
@@ -1437,7 +1425,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="102">
@@ -1447,7 +1435,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="103">
@@ -1457,7 +1445,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="104">
@@ -1467,7 +1455,7 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="105">
@@ -1477,7 +1465,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="106">
@@ -1487,7 +1475,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="107">
@@ -1507,7 +1495,7 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="109">
@@ -1517,7 +1505,7 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="110">
@@ -1527,7 +1515,7 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="111">
@@ -1537,7 +1525,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="112">
@@ -1547,7 +1535,7 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="113">
@@ -1557,7 +1545,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="114">
@@ -1567,7 +1555,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="115">
@@ -1587,7 +1575,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="117">
@@ -1597,7 +1585,7 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="118">
@@ -1607,7 +1595,7 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="119">
@@ -1637,7 +1625,7 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="122">
@@ -1657,7 +1645,7 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="124">
@@ -1667,7 +1655,7 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="125">
@@ -1677,7 +1665,7 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="126">
@@ -1687,7 +1675,7 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="127">
@@ -1697,7 +1685,7 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="128">
@@ -1707,7 +1695,7 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="129">
@@ -1717,7 +1705,7 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="130">
@@ -1737,7 +1725,7 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="132">
@@ -1757,7 +1745,7 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="134">
@@ -1767,7 +1755,7 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="135">
@@ -1777,7 +1765,7 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="136">
@@ -1787,7 +1775,7 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="137">
@@ -1807,7 +1795,7 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="139">
@@ -1817,7 +1805,7 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="140">
@@ -1827,7 +1815,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="141">
@@ -1847,7 +1835,7 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="143">
@@ -1857,7 +1845,7 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="144">
@@ -1877,7 +1865,7 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="146">
@@ -1887,7 +1875,7 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="147">
@@ -1897,7 +1885,7 @@
         </is>
       </c>
       <c r="B147" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="148">
@@ -1907,7 +1895,7 @@
         </is>
       </c>
       <c r="B148" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="149">
@@ -1917,7 +1905,7 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="150">
@@ -1927,7 +1915,7 @@
         </is>
       </c>
       <c r="B150" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="151">
@@ -1947,7 +1935,7 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="153">
@@ -1957,7 +1945,7 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="154">
@@ -1967,7 +1955,7 @@
         </is>
       </c>
       <c r="B154" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="155">
@@ -1977,7 +1965,7 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="156">
@@ -1987,7 +1975,7 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="157">
@@ -1997,7 +1985,7 @@
         </is>
       </c>
       <c r="B157" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="158">
@@ -2007,7 +1995,7 @@
         </is>
       </c>
       <c r="B158" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="159">
@@ -2017,7 +2005,7 @@
         </is>
       </c>
       <c r="B159" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="160">
@@ -2027,7 +2015,7 @@
         </is>
       </c>
       <c r="B160" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>